<commit_message>
update to raw data files
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/Erie/D100/ER 58 D100 Spring 2024 24GE02I93 Zoop.xlsx
+++ b/data/raw/GLNPO 2024 Spring/Erie/D100/ER 58 D100 Spring 2024 24GE02I93 Zoop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\Erie\D100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1787F44-8DB9-4FA0-9006-C86464016E12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FEFFFE-D6D6-4578-A67F-DE00F302B215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CD3F1934-A1BF-455C-95B0-483CCCA398C7}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="35" r:id="rId2"/>
+    <pivotCache cacheId="3" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3548" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3548" uniqueCount="92">
   <si>
     <t>SAMPLENUM</t>
   </si>
@@ -319,15 +319,12 @@
   <si>
     <t>Comment</t>
   </si>
-  <si>
-    <t>Paracyclops chiltoni</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,19 +350,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -375,7 +359,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -398,27 +382,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="22"/>
-      </left>
-      <right style="thin">
-        <color indexed="22"/>
-      </right>
-      <top style="thin">
-        <color indexed="22"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="22"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -430,13 +398,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 3" xfId="1" xr:uid="{56C4F9BF-5983-48B3-A5A9-CF1A0BAC112A}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -6309,7 +6273,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD10E709-52D3-4D22-AD0C-87F051213E05}" name="PivotTable1" cacheId="35" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD10E709-52D3-4D22-AD0C-87F051213E05}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="T3:X23" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
@@ -11900,7 +11864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>18</v>
       </c>
@@ -11931,8 +11895,8 @@
       <c r="J91" t="s">
         <v>24</v>
       </c>
-      <c r="K91" s="9" t="s">
-        <v>92</v>
+      <c r="K91" t="s">
+        <v>63</v>
       </c>
       <c r="L91" t="s">
         <v>64</v>
@@ -13917,7 +13881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>18</v>
       </c>
@@ -13948,8 +13912,8 @@
       <c r="J129" t="s">
         <v>24</v>
       </c>
-      <c r="K129" s="9" t="s">
-        <v>92</v>
+      <c r="K129" t="s">
+        <v>63</v>
       </c>
       <c r="L129" t="s">
         <v>64</v>
@@ -15457,7 +15421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>18</v>
       </c>
@@ -15488,8 +15452,8 @@
       <c r="J158" t="s">
         <v>24</v>
       </c>
-      <c r="K158" s="9" t="s">
-        <v>92</v>
+      <c r="K158" t="s">
+        <v>63</v>
       </c>
       <c r="L158" t="s">
         <v>64</v>
@@ -17047,7 +17011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>18</v>
       </c>
@@ -17078,8 +17042,8 @@
       <c r="J188" t="s">
         <v>24</v>
       </c>
-      <c r="K188" s="9" t="s">
-        <v>92</v>
+      <c r="K188" t="s">
+        <v>63</v>
       </c>
       <c r="L188" t="s">
         <v>64</v>
@@ -17153,7 +17117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>18</v>
       </c>
@@ -17184,8 +17148,8 @@
       <c r="J190" t="s">
         <v>24</v>
       </c>
-      <c r="K190" s="9" t="s">
-        <v>92</v>
+      <c r="K190" t="s">
+        <v>63</v>
       </c>
       <c r="L190" t="s">
         <v>64</v>
@@ -17683,7 +17647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>18</v>
       </c>
@@ -17714,8 +17678,8 @@
       <c r="J200" t="s">
         <v>24</v>
       </c>
-      <c r="K200" s="9" t="s">
-        <v>92</v>
+      <c r="K200" t="s">
+        <v>63</v>
       </c>
       <c r="L200" t="s">
         <v>64</v>
@@ -17842,7 +17806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>18</v>
       </c>
@@ -17873,8 +17837,8 @@
       <c r="J203" t="s">
         <v>24</v>
       </c>
-      <c r="K203" s="9" t="s">
-        <v>92</v>
+      <c r="K203" t="s">
+        <v>63</v>
       </c>
       <c r="L203" t="s">
         <v>64</v>
@@ -19432,7 +19396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>18</v>
       </c>
@@ -19463,8 +19427,8 @@
       <c r="J233" t="s">
         <v>24</v>
       </c>
-      <c r="K233" s="9" t="s">
-        <v>92</v>
+      <c r="K233" t="s">
+        <v>63</v>
       </c>
       <c r="L233" t="s">
         <v>64</v>
@@ -19591,7 +19555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>18</v>
       </c>
@@ -19622,8 +19586,8 @@
       <c r="J236" t="s">
         <v>24</v>
       </c>
-      <c r="K236" s="9" t="s">
-        <v>92</v>
+      <c r="K236" t="s">
+        <v>63</v>
       </c>
       <c r="L236" t="s">
         <v>64</v>
@@ -20280,7 +20244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>18</v>
       </c>
@@ -20311,8 +20275,8 @@
       <c r="J249" t="s">
         <v>24</v>
       </c>
-      <c r="K249" s="9" t="s">
-        <v>92</v>
+      <c r="K249" t="s">
+        <v>63</v>
       </c>
       <c r="L249" t="s">
         <v>64</v>
@@ -20439,7 +20403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>18</v>
       </c>
@@ -20470,8 +20434,8 @@
       <c r="J252" t="s">
         <v>24</v>
       </c>
-      <c r="K252" s="9" t="s">
-        <v>92</v>
+      <c r="K252" t="s">
+        <v>63</v>
       </c>
       <c r="L252" t="s">
         <v>64</v>
@@ -21234,7 +21198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>18</v>
       </c>
@@ -21265,8 +21229,8 @@
       <c r="J267" t="s">
         <v>24</v>
       </c>
-      <c r="K267" s="9" t="s">
-        <v>92</v>
+      <c r="K267" t="s">
+        <v>63</v>
       </c>
       <c r="L267" t="s">
         <v>64</v>
@@ -21658,7 +21622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>18</v>
       </c>
@@ -21689,8 +21653,8 @@
       <c r="J275" t="s">
         <v>24</v>
       </c>
-      <c r="K275" s="9" t="s">
-        <v>92</v>
+      <c r="K275" t="s">
+        <v>63</v>
       </c>
       <c r="L275" t="s">
         <v>64</v>
@@ -21764,7 +21728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="277" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>18</v>
       </c>
@@ -21795,8 +21759,8 @@
       <c r="J277" t="s">
         <v>24</v>
       </c>
-      <c r="K277" s="9" t="s">
-        <v>92</v>
+      <c r="K277" t="s">
+        <v>63</v>
       </c>
       <c r="L277" t="s">
         <v>64</v>
@@ -21811,7 +21775,7 @@
         <v>0.499</v>
       </c>
       <c r="P277" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q277">
         <v>1</v>
@@ -21870,7 +21834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>18</v>
       </c>
@@ -21901,8 +21865,8 @@
       <c r="J279" t="s">
         <v>24</v>
       </c>
-      <c r="K279" s="9" t="s">
-        <v>92</v>
+      <c r="K279" t="s">
+        <v>63</v>
       </c>
       <c r="L279" t="s">
         <v>64</v>
@@ -22082,7 +22046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>18</v>
       </c>
@@ -22113,8 +22077,8 @@
       <c r="J283" t="s">
         <v>24</v>
       </c>
-      <c r="K283" s="9" t="s">
-        <v>92</v>
+      <c r="K283" t="s">
+        <v>63</v>
       </c>
       <c r="L283" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
adjusting several raw files with edits
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/Erie/D100/ER 58 D100 Spring 2024 24GE02I93 Zoop.xlsx
+++ b/data/raw/GLNPO 2024 Spring/Erie/D100/ER 58 D100 Spring 2024 24GE02I93 Zoop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\Erie\D100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FEFFFE-D6D6-4578-A67F-DE00F302B215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29A8CA15-FD8C-4384-AC9F-97D2ECB57579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CD3F1934-A1BF-455C-95B0-483CCCA398C7}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId2"/>
+    <pivotCache cacheId="6" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -233,9 +233,6 @@
     <t xml:space="preserve">HAR </t>
   </si>
   <si>
-    <t>Paracyclops chittoni</t>
-  </si>
-  <si>
     <t>PARCHIT</t>
   </si>
   <si>
@@ -319,6 +316,9 @@
   <si>
     <t>Comment</t>
   </si>
+  <si>
+    <t>Paracyclops chiltoni</t>
+  </si>
 </sst>
 </file>
 
@@ -386,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -398,6 +398,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,7 +417,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gl Lab User" refreshedDate="45576.4552287037" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="288" xr:uid="{ABF5DA09-C83C-4748-AAD9-492EBA5A0F5F}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Chris Marshall" refreshedDate="46153.491465046296" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="288" xr:uid="{ABF5DA09-C83C-4748-AAD9-492EBA5A0F5F}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:R289" sheet="Sheet1"/>
   </cacheSource>
@@ -456,7 +457,7 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="COMBO" numFmtId="0">
-      <sharedItems count="18">
+      <sharedItems count="19">
         <s v="Leptodiaptomus minutus"/>
         <s v="Cyclops copepodites"/>
         <s v="Diaptomus copepodites"/>
@@ -469,12 +470,13 @@
         <s v="Skistodiaptomus oregonensis"/>
         <s v="Daphnia galeata mendotae"/>
         <s v="Harpacticoida spp."/>
-        <s v="Paracyclops chittoni"/>
+        <s v="Paracyclops chiltoni"/>
         <s v="Limnocalanus macrurus"/>
         <s v="Leptodora kindti"/>
         <s v="Daphnia retrocurva"/>
         <s v="Microcyclops rubellus"/>
         <s v="Daphnia spp."/>
+        <s v="Paracyclops chittoni" u="1"/>
       </sharedItems>
     </cacheField>
     <cacheField name="SPECCODE" numFmtId="0">
@@ -487,7 +489,7 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="LENGTH" numFmtId="0">
-      <sharedItems containsMixedTypes="1" containsNumber="1" minValue="0" maxValue="2.8330000000000002"/>
+      <sharedItems containsMixedTypes="1" containsNumber="1" minValue="0.28699999999999998" maxValue="2.8330000000000002"/>
     </cacheField>
     <cacheField name="SEX" numFmtId="0">
       <sharedItems/>
@@ -843,7 +845,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.4239999999999999"/>
     <s v="F"/>
     <n v="1"/>
@@ -923,7 +925,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.357"/>
     <s v="F"/>
     <n v="1"/>
@@ -1283,7 +1285,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.427"/>
     <s v="F"/>
     <n v="1"/>
@@ -1703,7 +1705,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.615"/>
     <s v="F"/>
     <n v="1"/>
@@ -1803,7 +1805,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.6160000000000001"/>
     <s v="F"/>
     <n v="1"/>
@@ -1843,9 +1845,9 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
-    <n v="0"/>
-    <s v="NA"/>
+    <s v="COP"/>
+    <n v="1.5469999999999999"/>
+    <s v="F"/>
     <n v="1"/>
     <m/>
   </r>
@@ -1863,7 +1865,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.548"/>
     <s v="F"/>
     <n v="1"/>
@@ -1983,7 +1985,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.542"/>
     <s v="F"/>
     <n v="1"/>
@@ -2143,7 +2145,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.605"/>
     <s v="F"/>
     <n v="1"/>
@@ -2303,7 +2305,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.74299999999999999"/>
     <s v="F"/>
     <n v="1"/>
@@ -2423,7 +2425,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.633"/>
     <s v="F"/>
     <n v="1"/>
@@ -2583,7 +2585,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.405"/>
     <s v="M"/>
     <n v="1"/>
@@ -2703,7 +2705,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.3460000000000001"/>
     <s v="F"/>
     <n v="1"/>
@@ -2723,7 +2725,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.5680000000000001"/>
     <s v="F"/>
     <n v="1"/>
@@ -2763,7 +2765,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.5509999999999999"/>
     <s v="F"/>
     <n v="1"/>
@@ -2963,7 +2965,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.5289999999999999"/>
     <s v="F"/>
     <n v="1"/>
@@ -3043,7 +3045,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.4339999999999999"/>
     <s v="F"/>
     <n v="1"/>
@@ -3063,7 +3065,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.68100000000000005"/>
     <s v="F"/>
     <n v="1"/>
@@ -3083,7 +3085,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.41"/>
     <s v="F"/>
     <n v="1"/>
@@ -3183,9 +3185,9 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.4730000000000001"/>
-    <s v="NA"/>
+    <s v="F"/>
     <n v="1"/>
     <m/>
   </r>
@@ -3243,7 +3245,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.321"/>
     <s v="M"/>
     <n v="1"/>
@@ -3263,7 +3265,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <n v="1.625"/>
     <s v="F"/>
     <n v="1"/>
@@ -3643,7 +3645,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.77300000000000002"/>
     <s v="F"/>
     <n v="1"/>
@@ -3663,7 +3665,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <s v="NA"/>
     <s v="M"/>
     <n v="2"/>
@@ -3683,7 +3685,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <s v="NA"/>
     <s v="F"/>
     <n v="13"/>
@@ -4063,7 +4065,7 @@
     <x v="16"/>
     <s v="MICRUBE"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.65300000000000002"/>
     <s v="M"/>
     <n v="1"/>
@@ -4243,7 +4245,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.749"/>
     <s v="F"/>
     <n v="1"/>
@@ -4283,7 +4285,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.78200000000000003"/>
     <s v="F"/>
     <n v="1"/>
@@ -4403,7 +4405,7 @@
     <x v="16"/>
     <s v="MICRUBE"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.55800000000000005"/>
     <s v="M"/>
     <n v="1"/>
@@ -4483,7 +4485,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.77"/>
     <s v="F"/>
     <n v="1"/>
@@ -4543,7 +4545,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.73399999999999999"/>
     <s v="F"/>
     <n v="1"/>
@@ -4624,7 +4626,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.42"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -4664,7 +4666,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.319"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -4883,7 +4885,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <s v="NA"/>
     <s v="M"/>
     <n v="13"/>
@@ -4903,7 +4905,7 @@
     <x v="7"/>
     <s v="LEOSICI"/>
     <s v="CAL"/>
-    <s v="CAL"/>
+    <s v="COP"/>
     <s v="NA"/>
     <s v="F"/>
     <n v="27"/>
@@ -5143,7 +5145,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.41399999999999998"/>
     <s v="F"/>
     <n v="1"/>
@@ -5203,7 +5205,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.46100000000000002"/>
     <s v="F"/>
     <n v="1"/>
@@ -5443,7 +5445,7 @@
     <x v="16"/>
     <s v="MICRUBE"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.56499999999999995"/>
     <s v="M"/>
     <n v="1"/>
@@ -5463,7 +5465,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.69599999999999995"/>
     <s v="F"/>
     <n v="1"/>
@@ -5523,7 +5525,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.60699999999999998"/>
     <s v="M"/>
     <n v="1"/>
@@ -5684,7 +5686,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.294"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -5823,7 +5825,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.73299999999999998"/>
     <s v="F"/>
     <n v="1"/>
@@ -5844,7 +5846,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.2629999999999999"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -5864,7 +5866,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.3169999999999999"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -5904,7 +5906,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.5009999999999999"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -5944,7 +5946,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.333"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -5964,7 +5966,7 @@
     <s v="MESEDAX"/>
     <s v="CYC"/>
     <s v="COP"/>
-    <n v="1.3160000000000001"/>
+    <s v="NA"/>
     <s v="F"/>
     <n v="1"/>
     <m/>
@@ -5983,7 +5985,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.56200000000000006"/>
     <s v="M"/>
     <n v="1"/>
@@ -6023,7 +6025,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.499"/>
     <s v="F"/>
     <n v="1"/>
@@ -6063,7 +6065,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.73099999999999998"/>
     <s v="F"/>
     <n v="1"/>
@@ -6143,7 +6145,7 @@
     <x v="12"/>
     <s v="PARCHIT"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <n v="0.76"/>
     <s v="F"/>
     <n v="1"/>
@@ -6243,7 +6245,7 @@
     <x v="16"/>
     <s v="MICRUBE"/>
     <s v="CYC"/>
-    <s v="CYC"/>
+    <s v="COP"/>
     <s v="NA"/>
     <s v="NA"/>
     <n v="0"/>
@@ -6273,7 +6275,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD10E709-52D3-4D22-AD0C-87F051213E05}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FD10E709-52D3-4D22-AD0C-87F051213E05}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="T3:X23" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
@@ -6294,7 +6296,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
-      <items count="19">
+      <items count="20">
         <item x="8"/>
         <item x="1"/>
         <item x="10"/>
@@ -6311,8 +6313,9 @@
         <item x="5"/>
         <item x="6"/>
         <item x="16"/>
+        <item m="1" x="18"/>
+        <item x="9"/>
         <item x="12"/>
-        <item x="9"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -6377,10 +6380,10 @@
       <x v="15"/>
     </i>
     <i>
-      <x v="16"/>
+      <x v="17"/>
     </i>
     <i>
-      <x v="17"/>
+      <x v="18"/>
     </i>
     <i t="grand">
       <x/>
@@ -6743,11 +6746,10 @@
     <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="4" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
@@ -6912,10 +6914,10 @@
         <v>1</v>
       </c>
       <c r="T3" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="U3" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
@@ -6971,19 +6973,19 @@
         <v>1</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U4" t="s">
         <v>21</v>
       </c>
       <c r="V4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="W4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="X4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
@@ -7041,16 +7043,16 @@
       <c r="T5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="U5">
+      <c r="U5" s="9">
         <v>3</v>
       </c>
-      <c r="V5">
-        <v>4</v>
-      </c>
-      <c r="W5">
+      <c r="V5" s="9">
+        <v>4</v>
+      </c>
+      <c r="W5" s="9">
         <v>9</v>
       </c>
-      <c r="X5">
+      <c r="X5" s="9">
         <v>16</v>
       </c>
     </row>
@@ -7109,13 +7111,14 @@
       <c r="T6" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="U6">
+      <c r="U6" s="9">
         <v>31</v>
       </c>
-      <c r="V6">
+      <c r="V6" s="9">
         <v>25</v>
       </c>
-      <c r="X6">
+      <c r="W6" s="9"/>
+      <c r="X6" s="9">
         <v>56</v>
       </c>
     </row>
@@ -7174,16 +7177,16 @@
       <c r="T7" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="U7">
+      <c r="U7" s="9">
         <v>2</v>
       </c>
-      <c r="V7">
+      <c r="V7" s="9">
         <v>0</v>
       </c>
-      <c r="W7">
+      <c r="W7" s="9">
         <v>2</v>
       </c>
-      <c r="X7">
+      <c r="X7" s="9">
         <v>4</v>
       </c>
     </row>
@@ -7240,18 +7243,18 @@
         <v>1</v>
       </c>
       <c r="T8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="U8">
-        <v>1</v>
-      </c>
-      <c r="V8">
+        <v>70</v>
+      </c>
+      <c r="U8" s="9">
+        <v>1</v>
+      </c>
+      <c r="V8" s="9">
         <v>5</v>
       </c>
-      <c r="W8">
-        <v>4</v>
-      </c>
-      <c r="X8">
+      <c r="W8" s="9">
+        <v>4</v>
+      </c>
+      <c r="X8" s="9">
         <v>10</v>
       </c>
     </row>
@@ -7308,18 +7311,18 @@
         <v>1</v>
       </c>
       <c r="T9" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="U9">
+        <v>76</v>
+      </c>
+      <c r="U9" s="9">
         <v>0</v>
       </c>
-      <c r="V9">
-        <v>1</v>
-      </c>
-      <c r="W9">
+      <c r="V9" s="9">
+        <v>1</v>
+      </c>
+      <c r="W9" s="9">
         <v>5</v>
       </c>
-      <c r="X9">
+      <c r="X9" s="9">
         <v>6</v>
       </c>
     </row>
@@ -7378,13 +7381,14 @@
       <c r="T10" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="U10">
+      <c r="U10" s="9">
         <v>53</v>
       </c>
-      <c r="V10">
+      <c r="V10" s="9">
         <v>42</v>
       </c>
-      <c r="X10">
+      <c r="W10" s="9"/>
+      <c r="X10" s="9">
         <v>95</v>
       </c>
     </row>
@@ -7443,16 +7447,16 @@
       <c r="T11" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="U11">
+      <c r="U11" s="9">
         <v>8</v>
       </c>
-      <c r="V11">
-        <v>4</v>
-      </c>
-      <c r="W11">
+      <c r="V11" s="9">
+        <v>4</v>
+      </c>
+      <c r="W11" s="9">
         <v>3</v>
       </c>
-      <c r="X11">
+      <c r="X11" s="9">
         <v>15</v>
       </c>
     </row>
@@ -7511,16 +7515,16 @@
       <c r="T12" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="U12">
-        <v>1</v>
-      </c>
-      <c r="V12">
-        <v>1</v>
-      </c>
-      <c r="W12">
+      <c r="U12" s="9">
+        <v>1</v>
+      </c>
+      <c r="V12" s="9">
+        <v>1</v>
+      </c>
+      <c r="W12" s="9">
         <v>8</v>
       </c>
-      <c r="X12">
+      <c r="X12" s="9">
         <v>10</v>
       </c>
     </row>
@@ -7579,13 +7583,14 @@
       <c r="T13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="U13">
+      <c r="U13" s="9">
         <v>53</v>
       </c>
-      <c r="V13">
+      <c r="V13" s="9">
         <v>60</v>
       </c>
-      <c r="X13">
+      <c r="W13" s="9"/>
+      <c r="X13" s="9">
         <v>113</v>
       </c>
     </row>
@@ -7644,13 +7649,14 @@
       <c r="T14" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="U14">
+      <c r="U14" s="9">
         <v>98</v>
       </c>
-      <c r="V14">
+      <c r="V14" s="9">
         <v>91</v>
       </c>
-      <c r="X14">
+      <c r="W14" s="9"/>
+      <c r="X14" s="9">
         <v>189</v>
       </c>
     </row>
@@ -7709,13 +7715,14 @@
       <c r="T15" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="U15">
+      <c r="U15" s="9">
         <v>35</v>
       </c>
-      <c r="V15">
+      <c r="V15" s="9">
         <v>40</v>
       </c>
-      <c r="X15">
+      <c r="W15" s="9"/>
+      <c r="X15" s="9">
         <v>75</v>
       </c>
     </row>
@@ -7772,18 +7779,18 @@
         <v>1</v>
       </c>
       <c r="T16" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="U16">
-        <v>1</v>
-      </c>
-      <c r="V16">
-        <v>1</v>
-      </c>
-      <c r="W16">
-        <v>1</v>
-      </c>
-      <c r="X16">
+        <v>67</v>
+      </c>
+      <c r="U16" s="9">
+        <v>1</v>
+      </c>
+      <c r="V16" s="9">
+        <v>1</v>
+      </c>
+      <c r="W16" s="9">
+        <v>1</v>
+      </c>
+      <c r="X16" s="9">
         <v>3</v>
       </c>
     </row>
@@ -7840,18 +7847,18 @@
         <v>1</v>
       </c>
       <c r="T17" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="U17">
+        <v>64</v>
+      </c>
+      <c r="U17" s="9">
         <v>3</v>
       </c>
-      <c r="V17">
+      <c r="V17" s="9">
         <v>7</v>
       </c>
-      <c r="W17">
+      <c r="W17" s="9">
         <v>9</v>
       </c>
-      <c r="X17">
+      <c r="X17" s="9">
         <v>19</v>
       </c>
     </row>
@@ -7910,16 +7917,16 @@
       <c r="T18" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="U18">
-        <v>19</v>
-      </c>
-      <c r="V18">
+      <c r="U18" s="9">
+        <v>19</v>
+      </c>
+      <c r="V18" s="9">
         <v>14</v>
       </c>
-      <c r="W18">
+      <c r="W18" s="9">
         <v>29</v>
       </c>
-      <c r="X18">
+      <c r="X18" s="9">
         <v>62</v>
       </c>
     </row>
@@ -7978,16 +7985,16 @@
       <c r="T19" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="U19">
+      <c r="U19" s="9">
         <v>13</v>
       </c>
-      <c r="V19">
+      <c r="V19" s="9">
         <v>9</v>
       </c>
-      <c r="W19">
+      <c r="W19" s="9">
         <v>17</v>
       </c>
-      <c r="X19">
+      <c r="X19" s="9">
         <v>39</v>
       </c>
     </row>
@@ -8044,18 +8051,18 @@
         <v>1</v>
       </c>
       <c r="T20" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="U20">
+        <v>74</v>
+      </c>
+      <c r="U20" s="9">
         <v>0</v>
       </c>
-      <c r="V20">
+      <c r="V20" s="9">
         <v>2</v>
       </c>
-      <c r="W20">
-        <v>1</v>
-      </c>
-      <c r="X20">
+      <c r="W20" s="9">
+        <v>1</v>
+      </c>
+      <c r="X20" s="9">
         <v>3</v>
       </c>
     </row>
@@ -8112,19 +8119,19 @@
         <v>1</v>
       </c>
       <c r="T21" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="U21">
+        <v>55</v>
+      </c>
+      <c r="U21" s="9">
         <v>3</v>
       </c>
-      <c r="V21">
-        <v>4</v>
-      </c>
-      <c r="W21">
-        <v>9</v>
-      </c>
-      <c r="X21">
-        <v>16</v>
+      <c r="V21" s="9">
+        <v>7</v>
+      </c>
+      <c r="W21" s="9">
+        <v>4</v>
+      </c>
+      <c r="X21" s="9">
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.3">
@@ -8180,19 +8187,19 @@
         <v>1</v>
       </c>
       <c r="T22" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="U22">
+        <v>91</v>
+      </c>
+      <c r="U22" s="9">
         <v>3</v>
       </c>
-      <c r="V22">
-        <v>7</v>
-      </c>
-      <c r="W22">
-        <v>4</v>
-      </c>
-      <c r="X22">
-        <v>14</v>
+      <c r="V22" s="9">
+        <v>4</v>
+      </c>
+      <c r="W22" s="9">
+        <v>9</v>
+      </c>
+      <c r="X22" s="9">
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.3">
@@ -8248,18 +8255,18 @@
         <v>1</v>
       </c>
       <c r="T23" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="U23">
+        <v>80</v>
+      </c>
+      <c r="U23" s="9">
         <v>327</v>
       </c>
-      <c r="V23">
+      <c r="V23" s="9">
         <v>317</v>
       </c>
-      <c r="W23">
+      <c r="W23" s="9">
         <v>101</v>
       </c>
-      <c r="X23">
+      <c r="X23" s="9">
         <v>745</v>
       </c>
     </row>
@@ -8422,10 +8429,10 @@
         <v>1</v>
       </c>
       <c r="T26" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="U26" s="8" t="s">
         <v>84</v>
-      </c>
-      <c r="U26" s="8" t="s">
-        <v>85</v>
       </c>
       <c r="V26" s="8">
         <v>1.002</v>
@@ -8485,7 +8492,7 @@
       </c>
       <c r="T27" s="8"/>
       <c r="U27" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="V27" s="8">
         <v>1.0009999999999999</v>
@@ -8544,10 +8551,10 @@
         <v>1</v>
       </c>
       <c r="T28" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="U28" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="V28" s="8">
         <v>1.0049999999999999</v>
@@ -8607,7 +8614,7 @@
       </c>
       <c r="T29" s="8"/>
       <c r="U29" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="V29" s="8">
         <v>0.996</v>
@@ -8666,10 +8673,10 @@
         <v>1</v>
       </c>
       <c r="T30" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="U30" s="8" t="s">
         <v>87</v>
-      </c>
-      <c r="U30" s="8" t="s">
-        <v>88</v>
       </c>
       <c r="V30" s="8"/>
     </row>
@@ -8726,10 +8733,10 @@
         <v>1</v>
       </c>
       <c r="T31" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="U31" s="8" t="s">
         <v>89</v>
-      </c>
-      <c r="U31" s="8" t="s">
-        <v>90</v>
       </c>
       <c r="V31" s="8"/>
     </row>
@@ -8786,7 +8793,7 @@
         <v>1</v>
       </c>
       <c r="T32" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="U32" s="8"/>
     </row>
@@ -11896,10 +11903,10 @@
         <v>24</v>
       </c>
       <c r="K91" t="s">
+        <v>91</v>
+      </c>
+      <c r="L91" t="s">
         <v>63</v>
-      </c>
-      <c r="L91" t="s">
-        <v>64</v>
       </c>
       <c r="M91" t="s">
         <v>48</v>
@@ -11949,10 +11956,10 @@
         <v>24</v>
       </c>
       <c r="K92" t="s">
+        <v>64</v>
+      </c>
+      <c r="L92" t="s">
         <v>65</v>
-      </c>
-      <c r="L92" t="s">
-        <v>66</v>
       </c>
       <c r="M92" t="s">
         <v>27</v>
@@ -12977,7 +12984,7 @@
         <v>1</v>
       </c>
       <c r="R111" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="112" spans="1:18" x14ac:dyDescent="0.3">
@@ -13171,13 +13178,13 @@
         <v>24</v>
       </c>
       <c r="K115" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L115" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="L115" s="3" t="s">
+      <c r="M115" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="M115" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="N115" s="3" t="s">
         <v>54</v>
@@ -13913,10 +13920,10 @@
         <v>24</v>
       </c>
       <c r="K129" t="s">
+        <v>91</v>
+      </c>
+      <c r="L129" t="s">
         <v>63</v>
-      </c>
-      <c r="L129" t="s">
-        <v>64</v>
       </c>
       <c r="M129" t="s">
         <v>48</v>
@@ -14072,13 +14079,13 @@
         <v>24</v>
       </c>
       <c r="K132" t="s">
+        <v>70</v>
+      </c>
+      <c r="L132" t="s">
         <v>71</v>
       </c>
-      <c r="L132" t="s">
+      <c r="M132" t="s">
         <v>72</v>
-      </c>
-      <c r="M132" t="s">
-        <v>73</v>
       </c>
       <c r="N132" t="s">
         <v>54</v>
@@ -14411,7 +14418,7 @@
         <v>1</v>
       </c>
       <c r="R138" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="139" spans="1:18" x14ac:dyDescent="0.3">
@@ -15082,10 +15089,10 @@
         <v>24</v>
       </c>
       <c r="K151" t="s">
+        <v>64</v>
+      </c>
+      <c r="L151" t="s">
         <v>65</v>
-      </c>
-      <c r="L151" t="s">
-        <v>66</v>
       </c>
       <c r="M151" t="s">
         <v>27</v>
@@ -15241,10 +15248,10 @@
         <v>24</v>
       </c>
       <c r="K154" t="s">
+        <v>64</v>
+      </c>
+      <c r="L154" t="s">
         <v>65</v>
-      </c>
-      <c r="L154" t="s">
-        <v>66</v>
       </c>
       <c r="M154" t="s">
         <v>27</v>
@@ -15453,10 +15460,10 @@
         <v>24</v>
       </c>
       <c r="K158" t="s">
+        <v>91</v>
+      </c>
+      <c r="L158" t="s">
         <v>63</v>
-      </c>
-      <c r="L158" t="s">
-        <v>64</v>
       </c>
       <c r="M158" t="s">
         <v>48</v>
@@ -15965,7 +15972,7 @@
         <v>-1</v>
       </c>
       <c r="E168" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F168">
         <v>4</v>
@@ -16018,7 +16025,7 @@
         <v>-1</v>
       </c>
       <c r="E169" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F169">
         <v>4</v>
@@ -16071,7 +16078,7 @@
         <v>-1</v>
       </c>
       <c r="E170" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F170">
         <v>4</v>
@@ -16124,7 +16131,7 @@
         <v>-1</v>
       </c>
       <c r="E171" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F171">
         <v>4</v>
@@ -16177,7 +16184,7 @@
         <v>-1</v>
       </c>
       <c r="E172" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F172">
         <v>4</v>
@@ -16230,7 +16237,7 @@
         <v>-1</v>
       </c>
       <c r="E173" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F173">
         <v>4</v>
@@ -16248,13 +16255,13 @@
         <v>24</v>
       </c>
       <c r="K173" t="s">
+        <v>70</v>
+      </c>
+      <c r="L173" t="s">
         <v>71</v>
       </c>
-      <c r="L173" t="s">
+      <c r="M173" t="s">
         <v>72</v>
-      </c>
-      <c r="M173" t="s">
-        <v>73</v>
       </c>
       <c r="N173" t="s">
         <v>54</v>
@@ -16283,7 +16290,7 @@
         <v>-1</v>
       </c>
       <c r="E174" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F174">
         <v>4</v>
@@ -16336,7 +16343,7 @@
         <v>-1</v>
       </c>
       <c r="E175" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F175">
         <v>4</v>
@@ -16389,7 +16396,7 @@
         <v>-1</v>
       </c>
       <c r="E176" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F176">
         <v>4</v>
@@ -16442,7 +16449,7 @@
         <v>-1</v>
       </c>
       <c r="E177" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F177">
         <v>4</v>
@@ -16460,13 +16467,13 @@
         <v>24</v>
       </c>
       <c r="K177" t="s">
+        <v>70</v>
+      </c>
+      <c r="L177" t="s">
         <v>71</v>
       </c>
-      <c r="L177" t="s">
+      <c r="M177" t="s">
         <v>72</v>
-      </c>
-      <c r="M177" t="s">
-        <v>73</v>
       </c>
       <c r="N177" t="s">
         <v>54</v>
@@ -16495,7 +16502,7 @@
         <v>-1</v>
       </c>
       <c r="E178" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F178">
         <v>4</v>
@@ -16548,7 +16555,7 @@
         <v>-1</v>
       </c>
       <c r="E179" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F179">
         <v>4</v>
@@ -16566,10 +16573,10 @@
         <v>24</v>
       </c>
       <c r="K179" t="s">
+        <v>74</v>
+      </c>
+      <c r="L179" t="s">
         <v>75</v>
-      </c>
-      <c r="L179" t="s">
-        <v>76</v>
       </c>
       <c r="M179" t="s">
         <v>48</v>
@@ -16601,7 +16608,7 @@
         <v>-1</v>
       </c>
       <c r="E180" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F180">
         <v>4</v>
@@ -16654,7 +16661,7 @@
         <v>-1</v>
       </c>
       <c r="E181" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F181">
         <v>4</v>
@@ -16707,7 +16714,7 @@
         <v>-1</v>
       </c>
       <c r="E182" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F182">
         <v>4</v>
@@ -16725,13 +16732,13 @@
         <v>24</v>
       </c>
       <c r="K182" t="s">
+        <v>70</v>
+      </c>
+      <c r="L182" t="s">
         <v>71</v>
       </c>
-      <c r="L182" t="s">
+      <c r="M182" t="s">
         <v>72</v>
-      </c>
-      <c r="M182" t="s">
-        <v>73</v>
       </c>
       <c r="N182" t="s">
         <v>54</v>
@@ -16760,7 +16767,7 @@
         <v>-1</v>
       </c>
       <c r="E183" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F183">
         <v>4</v>
@@ -16778,13 +16785,13 @@
         <v>24</v>
       </c>
       <c r="K183" t="s">
+        <v>70</v>
+      </c>
+      <c r="L183" t="s">
         <v>71</v>
       </c>
-      <c r="L183" t="s">
+      <c r="M183" t="s">
         <v>72</v>
-      </c>
-      <c r="M183" t="s">
-        <v>73</v>
       </c>
       <c r="N183" t="s">
         <v>54</v>
@@ -16813,7 +16820,7 @@
         <v>-1</v>
       </c>
       <c r="E184" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F184">
         <v>4</v>
@@ -16866,7 +16873,7 @@
         <v>-1</v>
       </c>
       <c r="E185" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F185">
         <v>4</v>
@@ -16884,13 +16891,13 @@
         <v>24</v>
       </c>
       <c r="K185" t="s">
+        <v>70</v>
+      </c>
+      <c r="L185" t="s">
         <v>71</v>
       </c>
-      <c r="L185" t="s">
+      <c r="M185" t="s">
         <v>72</v>
-      </c>
-      <c r="M185" t="s">
-        <v>73</v>
       </c>
       <c r="N185" t="s">
         <v>54</v>
@@ -16919,7 +16926,7 @@
         <v>-1</v>
       </c>
       <c r="E186" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F186">
         <v>4</v>
@@ -16937,10 +16944,10 @@
         <v>24</v>
       </c>
       <c r="K186" t="s">
+        <v>64</v>
+      </c>
+      <c r="L186" t="s">
         <v>65</v>
-      </c>
-      <c r="L186" t="s">
-        <v>66</v>
       </c>
       <c r="M186" t="s">
         <v>27</v>
@@ -16972,7 +16979,7 @@
         <v>-1</v>
       </c>
       <c r="E187" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F187">
         <v>4</v>
@@ -17025,7 +17032,7 @@
         <v>-1</v>
       </c>
       <c r="E188" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F188">
         <v>4</v>
@@ -17043,10 +17050,10 @@
         <v>24</v>
       </c>
       <c r="K188" t="s">
+        <v>91</v>
+      </c>
+      <c r="L188" t="s">
         <v>63</v>
-      </c>
-      <c r="L188" t="s">
-        <v>64</v>
       </c>
       <c r="M188" t="s">
         <v>48</v>
@@ -17078,7 +17085,7 @@
         <v>-1</v>
       </c>
       <c r="E189" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F189">
         <v>4</v>
@@ -17096,10 +17103,10 @@
         <v>24</v>
       </c>
       <c r="K189" t="s">
+        <v>64</v>
+      </c>
+      <c r="L189" t="s">
         <v>65</v>
-      </c>
-      <c r="L189" t="s">
-        <v>66</v>
       </c>
       <c r="M189" t="s">
         <v>27</v>
@@ -17131,7 +17138,7 @@
         <v>-1</v>
       </c>
       <c r="E190" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F190">
         <v>4</v>
@@ -17149,10 +17156,10 @@
         <v>24</v>
       </c>
       <c r="K190" t="s">
+        <v>91</v>
+      </c>
+      <c r="L190" t="s">
         <v>63</v>
-      </c>
-      <c r="L190" t="s">
-        <v>64</v>
       </c>
       <c r="M190" t="s">
         <v>48</v>
@@ -17184,7 +17191,7 @@
         <v>-1</v>
       </c>
       <c r="E191" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F191">
         <v>4</v>
@@ -17202,10 +17209,10 @@
         <v>24</v>
       </c>
       <c r="K191" t="s">
+        <v>64</v>
+      </c>
+      <c r="L191" t="s">
         <v>65</v>
-      </c>
-      <c r="L191" t="s">
-        <v>66</v>
       </c>
       <c r="M191" t="s">
         <v>27</v>
@@ -17237,7 +17244,7 @@
         <v>-1</v>
       </c>
       <c r="E192" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F192">
         <v>4</v>
@@ -17290,7 +17297,7 @@
         <v>-1</v>
       </c>
       <c r="E193" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F193">
         <v>4</v>
@@ -17308,10 +17315,10 @@
         <v>24</v>
       </c>
       <c r="K193" t="s">
+        <v>64</v>
+      </c>
+      <c r="L193" t="s">
         <v>65</v>
-      </c>
-      <c r="L193" t="s">
-        <v>66</v>
       </c>
       <c r="M193" t="s">
         <v>27</v>
@@ -17343,7 +17350,7 @@
         <v>-1</v>
       </c>
       <c r="E194" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F194">
         <v>4</v>
@@ -17361,10 +17368,10 @@
         <v>24</v>
       </c>
       <c r="K194" t="s">
+        <v>64</v>
+      </c>
+      <c r="L194" t="s">
         <v>65</v>
-      </c>
-      <c r="L194" t="s">
-        <v>66</v>
       </c>
       <c r="M194" t="s">
         <v>27</v>
@@ -17396,7 +17403,7 @@
         <v>-1</v>
       </c>
       <c r="E195" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F195">
         <v>4</v>
@@ -17449,7 +17456,7 @@
         <v>-1</v>
       </c>
       <c r="E196" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F196">
         <v>4</v>
@@ -17467,10 +17474,10 @@
         <v>24</v>
       </c>
       <c r="K196" t="s">
+        <v>74</v>
+      </c>
+      <c r="L196" t="s">
         <v>75</v>
-      </c>
-      <c r="L196" t="s">
-        <v>76</v>
       </c>
       <c r="M196" t="s">
         <v>48</v>
@@ -17502,7 +17509,7 @@
         <v>-1</v>
       </c>
       <c r="E197" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F197">
         <v>4</v>
@@ -17555,7 +17562,7 @@
         <v>-1</v>
       </c>
       <c r="E198" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F198">
         <v>4</v>
@@ -17608,7 +17615,7 @@
         <v>-1</v>
       </c>
       <c r="E199" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F199">
         <v>4</v>
@@ -17626,13 +17633,13 @@
         <v>24</v>
       </c>
       <c r="K199" t="s">
+        <v>67</v>
+      </c>
+      <c r="L199" t="s">
         <v>68</v>
       </c>
-      <c r="L199" t="s">
+      <c r="M199" t="s">
         <v>69</v>
-      </c>
-      <c r="M199" t="s">
-        <v>70</v>
       </c>
       <c r="N199" t="s">
         <v>54</v>
@@ -17661,7 +17668,7 @@
         <v>-1</v>
       </c>
       <c r="E200" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F200">
         <v>4</v>
@@ -17679,10 +17686,10 @@
         <v>24</v>
       </c>
       <c r="K200" t="s">
+        <v>91</v>
+      </c>
+      <c r="L200" t="s">
         <v>63</v>
-      </c>
-      <c r="L200" t="s">
-        <v>64</v>
       </c>
       <c r="M200" t="s">
         <v>48</v>
@@ -17714,7 +17721,7 @@
         <v>-1</v>
       </c>
       <c r="E201" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F201">
         <v>4</v>
@@ -17732,10 +17739,10 @@
         <v>24</v>
       </c>
       <c r="K201" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L201" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L201" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="M201" s="3" t="s">
         <v>59</v>
@@ -17767,7 +17774,7 @@
         <v>-1</v>
       </c>
       <c r="E202" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F202">
         <v>4</v>
@@ -17820,7 +17827,7 @@
         <v>-1</v>
       </c>
       <c r="E203" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F203">
         <v>4</v>
@@ -17838,10 +17845,10 @@
         <v>24</v>
       </c>
       <c r="K203" t="s">
+        <v>91</v>
+      </c>
+      <c r="L203" t="s">
         <v>63</v>
-      </c>
-      <c r="L203" t="s">
-        <v>64</v>
       </c>
       <c r="M203" t="s">
         <v>48</v>
@@ -17873,7 +17880,7 @@
         <v>-1</v>
       </c>
       <c r="E204" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F204">
         <v>4</v>
@@ -17926,7 +17933,7 @@
         <v>-1</v>
       </c>
       <c r="E205" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F205">
         <v>4</v>
@@ -17979,7 +17986,7 @@
         <v>-1</v>
       </c>
       <c r="E206" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F206">
         <v>4</v>
@@ -18032,7 +18039,7 @@
         <v>-1</v>
       </c>
       <c r="E207" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F207">
         <v>4</v>
@@ -18085,7 +18092,7 @@
         <v>-1</v>
       </c>
       <c r="E208" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F208">
         <v>4</v>
@@ -18138,7 +18145,7 @@
         <v>-1</v>
       </c>
       <c r="E209" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F209">
         <v>4</v>
@@ -18191,7 +18198,7 @@
         <v>-1</v>
       </c>
       <c r="E210" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F210">
         <v>4</v>
@@ -18244,7 +18251,7 @@
         <v>-1</v>
       </c>
       <c r="E211" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F211">
         <v>4</v>
@@ -18297,7 +18304,7 @@
         <v>-1</v>
       </c>
       <c r="E212" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F212">
         <v>4</v>
@@ -18315,10 +18322,10 @@
         <v>24</v>
       </c>
       <c r="K212" t="s">
+        <v>64</v>
+      </c>
+      <c r="L212" t="s">
         <v>65</v>
-      </c>
-      <c r="L212" t="s">
-        <v>66</v>
       </c>
       <c r="M212" t="s">
         <v>27</v>
@@ -18350,7 +18357,7 @@
         <v>-1</v>
       </c>
       <c r="E213" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F213">
         <v>4</v>
@@ -18368,10 +18375,10 @@
         <v>24</v>
       </c>
       <c r="K213" t="s">
+        <v>64</v>
+      </c>
+      <c r="L213" t="s">
         <v>65</v>
-      </c>
-      <c r="L213" t="s">
-        <v>66</v>
       </c>
       <c r="M213" t="s">
         <v>27</v>
@@ -18403,7 +18410,7 @@
         <v>-1</v>
       </c>
       <c r="E214" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F214">
         <v>4</v>
@@ -18456,7 +18463,7 @@
         <v>-1</v>
       </c>
       <c r="E215" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F215">
         <v>4</v>
@@ -18509,7 +18516,7 @@
         <v>-1</v>
       </c>
       <c r="E216" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F216">
         <v>4</v>
@@ -18562,7 +18569,7 @@
         <v>-1</v>
       </c>
       <c r="E217" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F217">
         <v>4</v>
@@ -18615,7 +18622,7 @@
         <v>-1</v>
       </c>
       <c r="E218" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F218">
         <v>4</v>
@@ -18668,7 +18675,7 @@
         <v>-1</v>
       </c>
       <c r="E219" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F219">
         <v>4</v>
@@ -18721,7 +18728,7 @@
         <v>-1</v>
       </c>
       <c r="E220" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F220">
         <v>4</v>
@@ -18774,7 +18781,7 @@
         <v>-1</v>
       </c>
       <c r="E221" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F221">
         <v>4</v>
@@ -18827,7 +18834,7 @@
         <v>-1</v>
       </c>
       <c r="E222" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F222">
         <v>4</v>
@@ -18880,7 +18887,7 @@
         <v>-1</v>
       </c>
       <c r="E223" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F223">
         <v>4</v>
@@ -18933,7 +18940,7 @@
         <v>-1</v>
       </c>
       <c r="E224" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F224">
         <v>2</v>
@@ -18951,10 +18958,10 @@
         <v>24</v>
       </c>
       <c r="K224" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L224" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L224" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="M224" s="3" t="s">
         <v>59</v>
@@ -18986,7 +18993,7 @@
         <v>-1</v>
       </c>
       <c r="E225" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F225">
         <v>2</v>
@@ -19004,10 +19011,10 @@
         <v>24</v>
       </c>
       <c r="K225" t="s">
+        <v>64</v>
+      </c>
+      <c r="L225" t="s">
         <v>65</v>
-      </c>
-      <c r="L225" t="s">
-        <v>66</v>
       </c>
       <c r="M225" t="s">
         <v>27</v>
@@ -19039,7 +19046,7 @@
         <v>-1</v>
       </c>
       <c r="E226" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F226">
         <v>2</v>
@@ -19092,7 +19099,7 @@
         <v>-1</v>
       </c>
       <c r="E227" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F227">
         <v>2</v>
@@ -19110,10 +19117,10 @@
         <v>24</v>
       </c>
       <c r="K227" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L227" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L227" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="M227" s="3" t="s">
         <v>59</v>
@@ -19145,7 +19152,7 @@
         <v>-1</v>
       </c>
       <c r="E228" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F228">
         <v>2</v>
@@ -19163,10 +19170,10 @@
         <v>24</v>
       </c>
       <c r="K228" t="s">
+        <v>64</v>
+      </c>
+      <c r="L228" t="s">
         <v>65</v>
-      </c>
-      <c r="L228" t="s">
-        <v>66</v>
       </c>
       <c r="M228" t="s">
         <v>27</v>
@@ -19198,7 +19205,7 @@
         <v>-1</v>
       </c>
       <c r="E229" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F229">
         <v>2</v>
@@ -19251,7 +19258,7 @@
         <v>-1</v>
       </c>
       <c r="E230" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F230">
         <v>2</v>
@@ -19304,7 +19311,7 @@
         <v>-1</v>
       </c>
       <c r="E231" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F231">
         <v>2</v>
@@ -19322,10 +19329,10 @@
         <v>24</v>
       </c>
       <c r="K231" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L231" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L231" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="M231" s="3" t="s">
         <v>59</v>
@@ -19357,7 +19364,7 @@
         <v>-1</v>
       </c>
       <c r="E232" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F232">
         <v>2</v>
@@ -19410,7 +19417,7 @@
         <v>-1</v>
       </c>
       <c r="E233" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F233">
         <v>2</v>
@@ -19428,10 +19435,10 @@
         <v>24</v>
       </c>
       <c r="K233" t="s">
+        <v>91</v>
+      </c>
+      <c r="L233" t="s">
         <v>63</v>
-      </c>
-      <c r="L233" t="s">
-        <v>64</v>
       </c>
       <c r="M233" t="s">
         <v>48</v>
@@ -19463,7 +19470,7 @@
         <v>-1</v>
       </c>
       <c r="E234" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F234">
         <v>2</v>
@@ -19516,7 +19523,7 @@
         <v>-1</v>
       </c>
       <c r="E235" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F235">
         <v>2</v>
@@ -19569,7 +19576,7 @@
         <v>-1</v>
       </c>
       <c r="E236" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F236">
         <v>2</v>
@@ -19587,10 +19594,10 @@
         <v>24</v>
       </c>
       <c r="K236" t="s">
+        <v>91</v>
+      </c>
+      <c r="L236" t="s">
         <v>63</v>
-      </c>
-      <c r="L236" t="s">
-        <v>64</v>
       </c>
       <c r="M236" t="s">
         <v>48</v>
@@ -19622,7 +19629,7 @@
         <v>-1</v>
       </c>
       <c r="E237" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F237">
         <v>2</v>
@@ -19640,10 +19647,10 @@
         <v>24</v>
       </c>
       <c r="K237" t="s">
+        <v>64</v>
+      </c>
+      <c r="L237" t="s">
         <v>65</v>
-      </c>
-      <c r="L237" t="s">
-        <v>66</v>
       </c>
       <c r="M237" t="s">
         <v>27</v>
@@ -19675,7 +19682,7 @@
         <v>-1</v>
       </c>
       <c r="E238" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F238">
         <v>2</v>
@@ -19728,7 +19735,7 @@
         <v>-1</v>
       </c>
       <c r="E239" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F239">
         <v>2</v>
@@ -19746,13 +19753,13 @@
         <v>24</v>
       </c>
       <c r="K239" t="s">
+        <v>70</v>
+      </c>
+      <c r="L239" t="s">
         <v>71</v>
       </c>
-      <c r="L239" t="s">
+      <c r="M239" t="s">
         <v>72</v>
-      </c>
-      <c r="M239" t="s">
-        <v>73</v>
       </c>
       <c r="N239" t="s">
         <v>54</v>
@@ -19781,7 +19788,7 @@
         <v>-1</v>
       </c>
       <c r="E240" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F240">
         <v>2</v>
@@ -19834,7 +19841,7 @@
         <v>-1</v>
       </c>
       <c r="E241" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F241">
         <v>2</v>
@@ -19852,10 +19859,10 @@
         <v>24</v>
       </c>
       <c r="K241" t="s">
+        <v>64</v>
+      </c>
+      <c r="L241" t="s">
         <v>65</v>
-      </c>
-      <c r="L241" t="s">
-        <v>66</v>
       </c>
       <c r="M241" t="s">
         <v>27</v>
@@ -19887,7 +19894,7 @@
         <v>-1</v>
       </c>
       <c r="E242" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F242">
         <v>2</v>
@@ -19905,10 +19912,10 @@
         <v>24</v>
       </c>
       <c r="K242" t="s">
+        <v>64</v>
+      </c>
+      <c r="L242" t="s">
         <v>65</v>
-      </c>
-      <c r="L242" t="s">
-        <v>66</v>
       </c>
       <c r="M242" t="s">
         <v>27</v>
@@ -19940,7 +19947,7 @@
         <v>-1</v>
       </c>
       <c r="E243" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F243">
         <v>2</v>
@@ -19993,7 +20000,7 @@
         <v>-1</v>
       </c>
       <c r="E244" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F244">
         <v>2</v>
@@ -20011,13 +20018,13 @@
         <v>24</v>
       </c>
       <c r="K244" t="s">
+        <v>70</v>
+      </c>
+      <c r="L244" t="s">
         <v>71</v>
       </c>
-      <c r="L244" t="s">
+      <c r="M244" t="s">
         <v>72</v>
-      </c>
-      <c r="M244" t="s">
-        <v>73</v>
       </c>
       <c r="N244" t="s">
         <v>54</v>
@@ -20046,7 +20053,7 @@
         <v>-1</v>
       </c>
       <c r="E245" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F245">
         <v>2</v>
@@ -20064,10 +20071,10 @@
         <v>24</v>
       </c>
       <c r="K245" t="s">
+        <v>64</v>
+      </c>
+      <c r="L245" t="s">
         <v>65</v>
-      </c>
-      <c r="L245" t="s">
-        <v>66</v>
       </c>
       <c r="M245" t="s">
         <v>27</v>
@@ -20099,7 +20106,7 @@
         <v>-1</v>
       </c>
       <c r="E246" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F246">
         <v>2</v>
@@ -20152,7 +20159,7 @@
         <v>-1</v>
       </c>
       <c r="E247" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F247">
         <v>2</v>
@@ -20205,7 +20212,7 @@
         <v>-1</v>
       </c>
       <c r="E248" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F248">
         <v>2</v>
@@ -20223,10 +20230,10 @@
         <v>24</v>
       </c>
       <c r="K248" t="s">
+        <v>74</v>
+      </c>
+      <c r="L248" t="s">
         <v>75</v>
-      </c>
-      <c r="L248" t="s">
-        <v>76</v>
       </c>
       <c r="M248" t="s">
         <v>48</v>
@@ -20258,7 +20265,7 @@
         <v>-1</v>
       </c>
       <c r="E249" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F249">
         <v>2</v>
@@ -20276,10 +20283,10 @@
         <v>24</v>
       </c>
       <c r="K249" t="s">
+        <v>91</v>
+      </c>
+      <c r="L249" t="s">
         <v>63</v>
-      </c>
-      <c r="L249" t="s">
-        <v>64</v>
       </c>
       <c r="M249" t="s">
         <v>48</v>
@@ -20311,7 +20318,7 @@
         <v>-1</v>
       </c>
       <c r="E250" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F250">
         <v>2</v>
@@ -20329,10 +20336,10 @@
         <v>24</v>
       </c>
       <c r="K250" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L250" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L250" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="M250" s="3" t="s">
         <v>59</v>
@@ -20364,7 +20371,7 @@
         <v>-1</v>
       </c>
       <c r="E251" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F251">
         <v>2</v>
@@ -20382,10 +20389,10 @@
         <v>24</v>
       </c>
       <c r="K251" t="s">
+        <v>64</v>
+      </c>
+      <c r="L251" t="s">
         <v>65</v>
-      </c>
-      <c r="L251" t="s">
-        <v>66</v>
       </c>
       <c r="M251" t="s">
         <v>27</v>
@@ -20417,7 +20424,7 @@
         <v>-1</v>
       </c>
       <c r="E252" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F252">
         <v>2</v>
@@ -20435,10 +20442,10 @@
         <v>24</v>
       </c>
       <c r="K252" t="s">
+        <v>91</v>
+      </c>
+      <c r="L252" t="s">
         <v>63</v>
-      </c>
-      <c r="L252" t="s">
-        <v>64</v>
       </c>
       <c r="M252" t="s">
         <v>48</v>
@@ -20470,7 +20477,7 @@
         <v>-1</v>
       </c>
       <c r="E253" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F253">
         <v>2</v>
@@ -20488,10 +20495,10 @@
         <v>24</v>
       </c>
       <c r="K253" t="s">
+        <v>64</v>
+      </c>
+      <c r="L253" t="s">
         <v>65</v>
-      </c>
-      <c r="L253" t="s">
-        <v>66</v>
       </c>
       <c r="M253" t="s">
         <v>27</v>
@@ -20523,7 +20530,7 @@
         <v>-1</v>
       </c>
       <c r="E254" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F254">
         <v>2</v>
@@ -20576,7 +20583,7 @@
         <v>-1</v>
       </c>
       <c r="E255" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F255">
         <v>2</v>
@@ -20629,7 +20636,7 @@
         <v>-1</v>
       </c>
       <c r="E256" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F256">
         <v>2</v>
@@ -20682,7 +20689,7 @@
         <v>-1</v>
       </c>
       <c r="E257" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F257">
         <v>2</v>
@@ -20735,7 +20742,7 @@
         <v>-1</v>
       </c>
       <c r="E258" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F258">
         <v>2</v>
@@ -20788,7 +20795,7 @@
         <v>-1</v>
       </c>
       <c r="E259" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F259">
         <v>2</v>
@@ -20806,13 +20813,13 @@
         <v>24</v>
       </c>
       <c r="K259" t="s">
+        <v>67</v>
+      </c>
+      <c r="L259" t="s">
         <v>68</v>
       </c>
-      <c r="L259" t="s">
+      <c r="M259" t="s">
         <v>69</v>
-      </c>
-      <c r="M259" t="s">
-        <v>70</v>
       </c>
       <c r="N259" t="s">
         <v>54</v>
@@ -20841,7 +20848,7 @@
         <v>-1</v>
       </c>
       <c r="E260" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F260">
         <v>2</v>
@@ -20894,7 +20901,7 @@
         <v>-1</v>
       </c>
       <c r="E261" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F261">
         <v>2</v>
@@ -20947,7 +20954,7 @@
         <v>-1</v>
       </c>
       <c r="E262" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F262">
         <v>2</v>
@@ -21000,7 +21007,7 @@
         <v>-1</v>
       </c>
       <c r="E263" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F263">
         <v>2</v>
@@ -21018,13 +21025,13 @@
         <v>24</v>
       </c>
       <c r="K263" t="s">
+        <v>70</v>
+      </c>
+      <c r="L263" t="s">
         <v>71</v>
       </c>
-      <c r="L263" t="s">
+      <c r="M263" t="s">
         <v>72</v>
-      </c>
-      <c r="M263" t="s">
-        <v>73</v>
       </c>
       <c r="N263" t="s">
         <v>54</v>
@@ -21053,7 +21060,7 @@
         <v>-1</v>
       </c>
       <c r="E264" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F264">
         <v>2</v>
@@ -21071,10 +21078,10 @@
         <v>24</v>
       </c>
       <c r="K264" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L264" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="L264" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="M264" s="3" t="s">
         <v>59</v>
@@ -21106,7 +21113,7 @@
         <v>-1</v>
       </c>
       <c r="E265" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F265">
         <v>2</v>
@@ -21159,7 +21166,7 @@
         <v>-1</v>
       </c>
       <c r="E266" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F266">
         <v>2</v>
@@ -21212,7 +21219,7 @@
         <v>-1</v>
       </c>
       <c r="E267" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F267">
         <v>2</v>
@@ -21230,10 +21237,10 @@
         <v>24</v>
       </c>
       <c r="K267" t="s">
+        <v>91</v>
+      </c>
+      <c r="L267" t="s">
         <v>63</v>
-      </c>
-      <c r="L267" t="s">
-        <v>64</v>
       </c>
       <c r="M267" t="s">
         <v>48</v>
@@ -21265,7 +21272,7 @@
         <v>-1</v>
       </c>
       <c r="E268" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F268">
         <v>2</v>
@@ -21318,7 +21325,7 @@
         <v>-1</v>
       </c>
       <c r="E269" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F269">
         <v>2</v>
@@ -21371,7 +21378,7 @@
         <v>-1</v>
       </c>
       <c r="E270" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F270">
         <v>2</v>
@@ -21424,7 +21431,7 @@
         <v>-1</v>
       </c>
       <c r="E271" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F271">
         <v>2</v>
@@ -21477,7 +21484,7 @@
         <v>-1</v>
       </c>
       <c r="E272" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F272">
         <v>2</v>
@@ -21495,10 +21502,10 @@
         <v>24</v>
       </c>
       <c r="K272" t="s">
+        <v>64</v>
+      </c>
+      <c r="L272" t="s">
         <v>65</v>
-      </c>
-      <c r="L272" t="s">
-        <v>66</v>
       </c>
       <c r="M272" t="s">
         <v>27</v>
@@ -21530,7 +21537,7 @@
         <v>-1</v>
       </c>
       <c r="E273" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F273">
         <v>2</v>
@@ -21583,7 +21590,7 @@
         <v>-1</v>
       </c>
       <c r="E274" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F274">
         <v>2</v>
@@ -21636,7 +21643,7 @@
         <v>-1</v>
       </c>
       <c r="E275" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F275">
         <v>2</v>
@@ -21654,10 +21661,10 @@
         <v>24</v>
       </c>
       <c r="K275" t="s">
+        <v>91</v>
+      </c>
+      <c r="L275" t="s">
         <v>63</v>
-      </c>
-      <c r="L275" t="s">
-        <v>64</v>
       </c>
       <c r="M275" t="s">
         <v>48</v>
@@ -21689,7 +21696,7 @@
         <v>-1</v>
       </c>
       <c r="E276" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F276">
         <v>2</v>
@@ -21707,13 +21714,13 @@
         <v>24</v>
       </c>
       <c r="K276" t="s">
+        <v>70</v>
+      </c>
+      <c r="L276" t="s">
         <v>71</v>
       </c>
-      <c r="L276" t="s">
+      <c r="M276" t="s">
         <v>72</v>
-      </c>
-      <c r="M276" t="s">
-        <v>73</v>
       </c>
       <c r="N276" t="s">
         <v>54</v>
@@ -21742,7 +21749,7 @@
         <v>-1</v>
       </c>
       <c r="E277" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F277">
         <v>2</v>
@@ -21760,10 +21767,10 @@
         <v>24</v>
       </c>
       <c r="K277" t="s">
+        <v>91</v>
+      </c>
+      <c r="L277" t="s">
         <v>63</v>
-      </c>
-      <c r="L277" t="s">
-        <v>64</v>
       </c>
       <c r="M277" t="s">
         <v>48</v>
@@ -21795,7 +21802,7 @@
         <v>-1</v>
       </c>
       <c r="E278" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F278">
         <v>2</v>
@@ -21848,7 +21855,7 @@
         <v>-1</v>
       </c>
       <c r="E279" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F279">
         <v>2</v>
@@ -21866,10 +21873,10 @@
         <v>24</v>
       </c>
       <c r="K279" t="s">
+        <v>91</v>
+      </c>
+      <c r="L279" t="s">
         <v>63</v>
-      </c>
-      <c r="L279" t="s">
-        <v>64</v>
       </c>
       <c r="M279" t="s">
         <v>48</v>
@@ -21901,7 +21908,7 @@
         <v>-1</v>
       </c>
       <c r="E280" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F280">
         <v>2</v>
@@ -21954,7 +21961,7 @@
         <v>-1</v>
       </c>
       <c r="E281" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F281">
         <v>2</v>
@@ -22007,7 +22014,7 @@
         <v>-1</v>
       </c>
       <c r="E282" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F282">
         <v>2</v>
@@ -22060,7 +22067,7 @@
         <v>-1</v>
       </c>
       <c r="E283" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F283">
         <v>2</v>
@@ -22078,10 +22085,10 @@
         <v>24</v>
       </c>
       <c r="K283" t="s">
+        <v>91</v>
+      </c>
+      <c r="L283" t="s">
         <v>63</v>
-      </c>
-      <c r="L283" t="s">
-        <v>64</v>
       </c>
       <c r="M283" t="s">
         <v>48</v>
@@ -22113,7 +22120,7 @@
         <v>-1</v>
       </c>
       <c r="E284" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F284">
         <v>2</v>
@@ -22166,7 +22173,7 @@
         <v>-1</v>
       </c>
       <c r="E285" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F285">
         <v>2</v>
@@ -22219,7 +22226,7 @@
         <v>-1</v>
       </c>
       <c r="E286" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F286">
         <v>2</v>
@@ -22272,7 +22279,7 @@
         <v>-1</v>
       </c>
       <c r="E287" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F287" s="4">
         <v>4</v>
@@ -22343,10 +22350,10 @@
         <v>24</v>
       </c>
       <c r="K288" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="L288" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="L288" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="M288" s="4" t="s">
         <v>48</v>
@@ -22396,10 +22403,10 @@
         <v>24</v>
       </c>
       <c r="K289" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="L289" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="L289" s="4" t="s">
-        <v>78</v>
       </c>
       <c r="M289" s="4" t="s">
         <v>59</v>

</xml_diff>